<commit_message>
AI entry: Paid salaries ₹3,20,000 (krish)
</commit_message>
<xml_diff>
--- a/AI_Financial_Report_Template.xlsx
+++ b/AI_Financial_Report_Template.xlsx
@@ -1,16 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profit &amp; Loss" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance Sheet" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flow" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transaction Log" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Profit &amp; Loss" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Balance Sheet" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Cash Flow" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Transaction Log" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="PL_2027_Q1" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="BS_2027_Q1" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="CF_2027_Q1" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -466,17 +469,13 @@
         <v/>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-      <c r="B5" t="inlineStr"/>
-    </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
           <t>Expenses</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -654,7 +653,6 @@
           <t>ASSETS</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -753,7 +751,6 @@
           <t>EQUITY</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -781,7 +778,6 @@
           <t>LIABILITIES</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -856,7 +852,6 @@
           <t>Operating Activities</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -874,7 +869,6 @@
           <t>Investing Activities</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -892,7 +886,6 @@
           <t>Financing Activities</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -936,44 +929,646 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>Fiscal Year</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Quarter</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>Date</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Original Transaction</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Statement</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Line Item</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Operation</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-07-16T05:06:50.725087+00:00</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Paid salaries ₹3,20,000</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Profit &amp; Loss</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Employee Benefits Expense</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>320000</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-07-16T05:06:50.732099+00:00</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Paid salaries ₹3,20,000</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Balance Sheet</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Cash &amp; Cash Equivalents</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>320000</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>subtract</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Particulars</t>
+        </is>
+      </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Original Transaction</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Statement</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Line Item</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Operation</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Revenue From Operations</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Other Income</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Total Income</t>
+        </is>
+      </c>
+      <c r="B4">
+        <f>SUM(B2:B3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5"/>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Cost of Materials Consumed</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Purchases of Stock-in-Trade</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Changes in Inventories</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Employee Benefits Expense</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>320000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Finance Costs</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Depreciation &amp; Amortisation Expenses</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Other Expenses</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Total Expenses</t>
+        </is>
+      </c>
+      <c r="B14">
+        <f>SUM(B7:B13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Profit Before Exceptional Items &amp; Tax</t>
+        </is>
+      </c>
+      <c r="B15">
+        <f>B4-B14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Exceptional Items</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Profit Before Tax</t>
+        </is>
+      </c>
+      <c r="B17">
+        <f>B15-B16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Current Tax</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Deferred Tax</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Profit After Tax</t>
+        </is>
+      </c>
+      <c r="B20">
+        <f>B17-B18-B19</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Particulars</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ASSETS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Property, Plant &amp; Equipment</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Right of Use Assets</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Investment Property</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Other Intangible Assets</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Inventories</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Trade Receivables</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Cash &amp; Cash Equivalents</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>-320000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Other Current Assets</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TOTAL ASSETS</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>SUM(B3:B9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>EQUITY</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Equity Share Capital</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Other Equity</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>LIABILITIES</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Borrowings</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Trade Payables</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Other Current Liabilities</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>TOTAL EQUITY &amp; LIABILITIES</t>
+        </is>
+      </c>
+      <c r="B19">
+        <f>SUM(B12:B17)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Particulars</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Operating Activities</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Net Cash from Operating</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Investing Activities</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Net Cash from Investing</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Financing Activities</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Net Cash from Financing</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Opening Cash</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Closing Cash</t>
+        </is>
+      </c>
+      <c r="B9">
+        <f>SUM(B2,B4,B6,B7)</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AI entry: Purchased raw materials ₹8 lakh (krish)
</commit_message>
<xml_diff>
--- a/AI_Financial_Report_Template.xlsx
+++ b/AI_Financial_Report_Template.xlsx
@@ -469,7 +469,6 @@
         <v/>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
@@ -929,7 +928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1060,6 +1059,92 @@
         </is>
       </c>
       <c r="I3" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-07-16T05:07:10.947757+00:00</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Purchased raw materials ₹8 lakh</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Balance Sheet</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Inventories</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>800000</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-07-16T05:07:10.954579+00:00</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Purchased raw materials ₹8 lakh</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Profit &amp; Loss</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Cost of Materials Consumed</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>800000</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
@@ -1137,7 +1222,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>800000</v>
       </c>
     </row>
     <row r="8">
@@ -1354,7 +1439,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>800000</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
AI entry: SOLD LAPTOPS WORTH 20 CRORES (krish)
</commit_message>
<xml_diff>
--- a/AI_Financial_Report_Template.xlsx
+++ b/AI_Financial_Report_Template.xlsx
@@ -928,7 +928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1145,6 +1145,92 @@
         </is>
       </c>
       <c r="I5" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-07-16T05:07:26.250581+00:00</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>SOLD LAPTOPS WORTH 20 CRORES</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Profit &amp; Loss</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Revenue From Operations</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>200000000</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-07-16T05:07:26.262141+00:00</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>SOLD LAPTOPS WORTH 20 CRORES</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Balance Sheet</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Trade Receivables</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>200000000</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
@@ -1183,7 +1269,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>200000000</v>
       </c>
     </row>
     <row r="3">
@@ -1207,7 +1293,6 @@
         <v/>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
@@ -1449,7 +1534,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>200000000</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
AI entry: GOT AN INTEREST OF 5 LAKHS FROM BANK (krish)
</commit_message>
<xml_diff>
--- a/AI_Financial_Report_Template.xlsx
+++ b/AI_Financial_Report_Template.xlsx
@@ -928,7 +928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1231,6 +1231,92 @@
         </is>
       </c>
       <c r="I7" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-07-16T05:08:03.302303+00:00</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>GOT AN INTEREST OF 5 LAKHS FROM BANK</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Profit &amp; Loss</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Other Income</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>500000</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-07-16T05:08:03.314266+00:00</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>GOT AN INTEREST OF 5 LAKHS FROM BANK</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Balance Sheet</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Cash &amp; Cash Equivalents</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>500000</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
@@ -1279,7 +1365,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>500000</v>
       </c>
     </row>
     <row r="4">
@@ -1544,7 +1630,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-320000</v>
+        <v>180000</v>
       </c>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
AI entry: sold worht 20000000 (krish)
</commit_message>
<xml_diff>
--- a/AI_Financial_Report_Template.xlsx
+++ b/AI_Financial_Report_Template.xlsx
@@ -14,6 +14,9 @@
     <sheet name="PL_2027_Q1" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="BS_2027_Q1" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="CF_2027_Q1" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="PL_2027_Q2" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="BS_2027_Q2" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="CF_2027_Q2" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -625,6 +628,104 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Particulars</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Operating Activities</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Net Cash from Operating</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Investing Activities</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Net Cash from Investing</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Financing Activities</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Net Cash from Financing</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Opening Cash</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Closing Cash</t>
+        </is>
+      </c>
+      <c r="B9">
+        <f>SUM(B2,B4,B6,B7)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -928,7 +1029,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1317,6 +1418,49 @@
         </is>
       </c>
       <c r="I9" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-07-16T05:15:51.818059+00:00</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>sold worht 20000000</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Profit &amp; Loss</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Revenue From Operations</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
@@ -1830,4 +1974,412 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Particulars</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Revenue From Operations</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>20000000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Other Income</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Total Income</t>
+        </is>
+      </c>
+      <c r="B4">
+        <f>SUM(B2:B3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5"/>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Cost of Materials Consumed</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Purchases of Stock-in-Trade</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Changes in Inventories</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Employee Benefits Expense</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Finance Costs</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Depreciation &amp; Amortisation Expenses</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Other Expenses</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Total Expenses</t>
+        </is>
+      </c>
+      <c r="B14">
+        <f>SUM(B7:B13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Profit Before Exceptional Items &amp; Tax</t>
+        </is>
+      </c>
+      <c r="B15">
+        <f>B4-B14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Exceptional Items</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Profit Before Tax</t>
+        </is>
+      </c>
+      <c r="B17">
+        <f>B15-B16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Current Tax</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Deferred Tax</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Profit After Tax</t>
+        </is>
+      </c>
+      <c r="B20">
+        <f>B17-B18-B19</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Particulars</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ASSETS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Property, Plant &amp; Equipment</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Right of Use Assets</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Investment Property</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Other Intangible Assets</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Inventories</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Trade Receivables</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Cash &amp; Cash Equivalents</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Other Current Assets</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TOTAL ASSETS</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>SUM(B3:B9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>EQUITY</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Equity Share Capital</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Other Equity</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>LIABILITIES</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Borrowings</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Trade Payables</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Other Current Liabilities</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>TOTAL EQUITY &amp; LIABILITIES</t>
+        </is>
+      </c>
+      <c r="B19">
+        <f>SUM(B12:B17)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
AI entry: paid tax of 50 lakhs (krish)
</commit_message>
<xml_diff>
--- a/AI_Financial_Report_Template.xlsx
+++ b/AI_Financial_Report_Template.xlsx
@@ -1029,7 +1029,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1461,6 +1461,92 @@
         </is>
       </c>
       <c r="I10" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-07-16T05:24:39.877652+00:00</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>paid tax of 50 lakhs</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Profit &amp; Loss</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Current Tax</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2026-07-16T05:24:39.892719+00:00</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>paid tax of 50 lakhs</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Balance Sheet</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Cash &amp; Cash Equivalents</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>subtract</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
@@ -2156,7 +2242,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0</v>
+        <v>5000000</v>
       </c>
     </row>
     <row r="19">
@@ -2280,7 +2366,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>-5000000</v>
       </c>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
Undo last transaction for Q1 FY2027
</commit_message>
<xml_diff>
--- a/AI_Financial_Report_Template.xlsx
+++ b/AI_Financial_Report_Template.xlsx
@@ -1029,7 +1029,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Applied</t>
+          <t>Reversed</t>
         </is>
       </c>
     </row>
@@ -1549,6 +1549,49 @@
       <c r="I12" t="inlineStr">
         <is>
           <t>Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-07-16T05:25:41.613193+00:00</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>UNDO: GOT AN INTEREST OF 5 LAKHS FROM BANK</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Balance Sheet</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Cash &amp; Cash Equivalents</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>500000</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>subtract</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Applied (undo)</t>
         </is>
       </c>
     </row>
@@ -1860,7 +1903,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>180000</v>
+        <v>-320000</v>
       </c>
     </row>
     <row r="10">
@@ -2114,7 +2157,6 @@
         <v/>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
AI entry: earned 30000 (krish)
</commit_message>
<xml_diff>
--- a/AI_Financial_Report_Template.xlsx
+++ b/AI_Financial_Report_Template.xlsx
@@ -1029,7 +1029,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1721,6 +1721,49 @@
       <c r="I16" t="inlineStr">
         <is>
           <t>Applied (undo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2026-07-16T05:27:59.115629+00:00</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>earned 30000</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Profit &amp; Loss</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Revenue From Operations</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>30000</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Applied</t>
         </is>
       </c>
     </row>
@@ -1757,7 +1800,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Log rejected transaction (krish)
</commit_message>
<xml_diff>
--- a/AI_Financial_Report_Template.xlsx
+++ b/AI_Financial_Report_Template.xlsx
@@ -1029,7 +1029,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1764,6 +1764,49 @@
       <c r="I17" t="inlineStr">
         <is>
           <t>Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2026-07-16T05:28:09.781263+00:00</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>lost 20000</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Rejected: Please specify the nature of the loss (e.g., theft, bad debt, asset impairment) so I can classify it correctly under Other Expenses or Exceptional Items.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
AI entry: bad debt 20000 (krish)
</commit_message>
<xml_diff>
--- a/AI_Financial_Report_Template.xlsx
+++ b/AI_Financial_Report_Template.xlsx
@@ -1029,7 +1029,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1850,6 +1850,92 @@
       <c r="I19" t="inlineStr">
         <is>
           <t>Rejected: Please provide the specific amount for the bad debt write-off.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2026-07-16T05:28:36.469500+00:00</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>bad debt 20000</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Profit &amp; Loss</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Other Expenses</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>20000</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2026-07-16T05:28:36.485515+00:00</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>bad debt 20000</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Balance Sheet</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Trade Receivables</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>20000</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>subtract</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Applied</t>
         </is>
       </c>
     </row>
@@ -1910,6 +1996,7 @@
         <v/>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
@@ -1984,7 +2071,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="14">
@@ -2151,7 +2238,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>-20000</v>
       </c>
     </row>
     <row r="9">

</xml_diff>